<commit_message>
Normalize stray ampullaofvater -> ampulla_of_vater
v3_multi_type_residue.txt and v3_multi_type_variant_file.txt had 6 and 18
rows respectively that still carried the raw v3 tumor-type name
'ampullaofvater' because normalize_data.py's TUMOR_TYPE_MAP was missing
that entry.

Add the mapping, and add fix_ampullaofvater.py to apply it in place
(normalize_data.py is a one-shot rebuild from a v2 baseline and backup,
so re-running it would be destructive).

Regenerate hotspots_v3.xlsx so the Samples column uses the canonical
name. All 30 tumor-type names in the xlsx Samples column now match
v2_multi_type_residue.txt.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/webapp/src/main/resources/static/files/hotspots_v3.xlsx
+++ b/webapp/src/main/resources/static/files/hotspots_v3.xlsx
@@ -2862,7 +2862,7 @@
       </c>
       <c r="Y28" s="2" t="inlineStr">
         <is>
-          <t>ampullaofvater:1|bladder:1|bowel:4</t>
+          <t>ampulla_of_vater:1|bladder:1|bowel:4</t>
         </is>
       </c>
       <c r="Z28" s="2" t="n"/>
@@ -9169,7 +9169,7 @@
       </c>
       <c r="Y101" s="2" t="inlineStr">
         <is>
-          <t>ampullaofvater:1|biliary_tract:1|bladder:1|bowel:1|liver:1|lung:2|skin:1|unk:1|uterus:1</t>
+          <t>ampulla_of_vater:1|biliary_tract:1|bladder:1|bowel:1|liver:1|lung:2|skin:1|unk:1|uterus:1</t>
         </is>
       </c>
       <c r="Z101" s="2" t="n"/>
@@ -10370,7 +10370,7 @@
       </c>
       <c r="Y115" s="2" t="inlineStr">
         <is>
-          <t>ampullaofvater:1|biliary_tract:1|bowel:1|stomach:2|lung:1|pancreas:4|uterus:1</t>
+          <t>ampulla_of_vater:1|biliary_tract:1|bowel:1|stomach:2|lung:1|pancreas:4|uterus:1</t>
         </is>
       </c>
       <c r="Z115" s="2" t="n"/>
@@ -10805,7 +10805,7 @@
       </c>
       <c r="Y120" s="2" t="inlineStr">
         <is>
-          <t>ampullaofvater:1|bowel:4|lung:1|pancreas:2|unk:1</t>
+          <t>ampulla_of_vater:1|bowel:4|lung:1|pancreas:2|unk:1</t>
         </is>
       </c>
       <c r="Z120" s="2" t="n"/>
@@ -13721,7 +13721,7 @@
       </c>
       <c r="Y154" s="2" t="inlineStr">
         <is>
-          <t>ampullaofvater:1|bowel:1|breast:2|brain:2|stomach:1|head_neck:2|liver:2|lung:12|blood:1|ovary:2|pleura:1|thyroid:1|unk:1|uterus:3|vulva:1</t>
+          <t>ampulla_of_vater:1|bowel:1|breast:2|brain:2|stomach:1|head_neck:2|liver:2|lung:12|blood:1|ovary:2|pleura:1|thyroid:1|unk:1|uterus:3|vulva:1</t>
         </is>
       </c>
       <c r="Z154" s="2" t="n"/>
@@ -13894,7 +13894,7 @@
       </c>
       <c r="Y156" s="2" t="inlineStr">
         <is>
-          <t>ampullaofvater:1|bladder:3|bowel:3|breast:2|brain:1|stomach:1|head_neck:5|lung:11|ovary:1|pancreas:2|unk:4|uterus:3|vulva:1</t>
+          <t>ampulla_of_vater:1|bladder:3|bowel:3|breast:2|brain:1|stomach:1|head_neck:5|lung:11|ovary:1|pancreas:2|unk:4|uterus:3|vulva:1</t>
         </is>
       </c>
       <c r="Z156" s="2" t="n"/>
@@ -14773,7 +14773,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:1|kidney:1|blood:1|ovary:1|prostate:1|thymus:1|unk:1</t>
         </is>
@@ -14802,7 +14802,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="0" t="inlineStr">
         <is>
           <t>bowel:2|blood:1|prostate:3|unk:1|uterus:4</t>
         </is>
@@ -14831,7 +14831,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="0" t="inlineStr">
         <is>
           <t>bladder:2|stomach:1|lung:1|blood:3|unk:2</t>
         </is>
@@ -14860,7 +14860,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:3|breast:1|brain:1|lung:4|blood:1|pancreas:1|soft_tissue:1</t>
         </is>
@@ -14885,7 +14885,7 @@
         <v>11.8</v>
       </c>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="0" t="inlineStr">
         <is>
           <t>bladder:2|breast:1|lung:3|blood:1|prostate:1|skin:1|thyroid:1</t>
         </is>
@@ -14914,7 +14914,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bladder:1|kidney:3|pleura:2</t>
         </is>
@@ -14943,7 +14943,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:2|bladder:1|eye:1|kidney:3|liver:1|lung:1|prostate:1|uterus:1</t>
         </is>
@@ -14972,7 +14972,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:2|stomach:1|head_neck:1|lung:5|blood:2|testis:1|uterus:2</t>
         </is>
@@ -15001,7 +15001,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:5|blood:3|skin:2</t>
         </is>
@@ -15026,7 +15026,7 @@
         <v>3.5</v>
       </c>
       <c r="F11" s="6" t="n"/>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="0" t="inlineStr">
         <is>
           <t>breast:6|blood:1</t>
         </is>
@@ -15051,7 +15051,7 @@
         <v>7.9</v>
       </c>
       <c r="F12" s="6" t="n"/>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:3|stomach:2</t>
         </is>
@@ -15080,7 +15080,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:2|stomach:4|uterus:1</t>
         </is>
@@ -15109,7 +15109,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="0" t="inlineStr">
         <is>
           <t>bowel:3|breast:3|stomach:1|uterus:5</t>
         </is>
@@ -15138,7 +15138,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:1|stomach:1|blood:1|ovary:2|prostate:5|skin:2</t>
         </is>
@@ -15167,7 +15167,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|breast:3|stomach:1|liver:2|lung:3|pancreas:3|skin:10|unk:1</t>
         </is>
@@ -15196,7 +15196,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:1|stomach:3|head_neck:3|lung:4|blood:5|skin:2|unk:1|uterus:1</t>
         </is>
@@ -15225,7 +15225,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="0" t="inlineStr">
         <is>
           <t>bowel:2|brain:1|blood:3|thyroid:3|uterus:8</t>
         </is>
@@ -15254,7 +15254,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="0" t="inlineStr">
         <is>
           <t>breast:1|lung:3|soft_tissue:5|unk:1|uterus:2</t>
         </is>
@@ -15283,7 +15283,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:1|brain:1|lung:1|blood:7|peritoneum:1|prostate:1|thyroid:1|unk:1|uterus:1</t>
         </is>
@@ -15312,7 +15312,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="0" t="inlineStr">
         <is>
           <t>lung:5</t>
         </is>
@@ -15341,7 +15341,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:2|lung:8|blood:1|soft_tissue:1</t>
         </is>
@@ -15370,7 +15370,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="0" t="inlineStr">
         <is>
           <t>lung:13</t>
         </is>
@@ -15399,7 +15399,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="0" t="inlineStr">
         <is>
           <t>lung:7</t>
         </is>
@@ -15428,7 +15428,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:3|stomach:2|head_neck:1|ovary:1|unk:1|uterus:1</t>
         </is>
@@ -15453,7 +15453,7 @@
         <v>7.9</v>
       </c>
       <c r="F26" s="6" t="n"/>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="0" t="inlineStr">
         <is>
           <t>bowel:4|pancreas:1|uterus:1</t>
         </is>
@@ -15478,7 +15478,7 @@
         <v>10.8</v>
       </c>
       <c r="F27" s="6" t="n"/>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="0" t="inlineStr">
         <is>
           <t>bladder:3|bowel:2|stomach:1|uterus:2</t>
         </is>
@@ -15507,9 +15507,9 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>ampullaofvater:1|bladder:1|bowel:4</t>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>ampulla_of_vater:1|bladder:1|bowel:4</t>
         </is>
       </c>
     </row>
@@ -15536,7 +15536,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="0" t="inlineStr">
         <is>
           <t>bladder:11</t>
         </is>
@@ -15561,7 +15561,7 @@
         <v>19.8</v>
       </c>
       <c r="F30" s="6" t="n"/>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="0" t="inlineStr">
         <is>
           <t>bladder:6</t>
         </is>
@@ -15590,7 +15590,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="0" t="inlineStr">
         <is>
           <t>breast:3|skin:1|uterus:4</t>
         </is>
@@ -15615,7 +15615,7 @@
         <v>6.15</v>
       </c>
       <c r="F32" s="6" t="n"/>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="0" t="inlineStr">
         <is>
           <t>bowel:1|stomach:1|ovary:1|uterus:5</t>
         </is>
@@ -15640,7 +15640,7 @@
         <v>11.15</v>
       </c>
       <c r="F33" s="6" t="n"/>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="0" t="inlineStr">
         <is>
           <t>bowel:7</t>
         </is>
@@ -15669,7 +15669,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:3</t>
         </is>
@@ -15698,7 +15698,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="0" t="inlineStr">
         <is>
           <t>bladder:3|bowel:1|breast:4|cervix:1|brain:1|stomach:1|lung:3|ovary:1|uterus:6</t>
         </is>
@@ -15723,7 +15723,7 @@
         <v>7.9</v>
       </c>
       <c r="F36" s="6" t="n"/>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="0" t="inlineStr">
         <is>
           <t>bladder:1|breast:1|kidney:1|prostate:4</t>
         </is>
@@ -15752,7 +15752,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" s="0" t="inlineStr">
         <is>
           <t>breast:5|blood:2|soft_tissue:2</t>
         </is>
@@ -15777,7 +15777,7 @@
         <v>9.699999999999999</v>
       </c>
       <c r="F38" s="6" t="n"/>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="0" t="inlineStr">
         <is>
           <t>kidney:1|liver:1|lung:7</t>
         </is>
@@ -15802,7 +15802,7 @@
         <v>7.45</v>
       </c>
       <c r="F39" s="6" t="n"/>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="0" t="inlineStr">
         <is>
           <t>head_neck:1|liver:1|lung:5|unk:1</t>
         </is>
@@ -15831,7 +15831,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="0" t="inlineStr">
         <is>
           <t>bowel:2|stomach:1|liver:1|lung:10</t>
         </is>
@@ -15856,7 +15856,7 @@
         <v>8.949999999999999</v>
       </c>
       <c r="F41" s="6" t="n"/>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="0" t="inlineStr">
         <is>
           <t>bladder:1|cervix:1|head_neck:1|lung:9</t>
         </is>
@@ -15881,7 +15881,7 @@
         <v>11.6</v>
       </c>
       <c r="F42" s="6" t="n"/>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="0" t="inlineStr">
         <is>
           <t>bladder:1|eye:1|lung:6|unk:2|uterus:3</t>
         </is>
@@ -15906,7 +15906,7 @@
         <v>12.3</v>
       </c>
       <c r="F43" s="6" t="n"/>
-      <c r="G43" t="inlineStr">
+      <c r="G43" s="0" t="inlineStr">
         <is>
           <t>stomach:1|kidney:2|liver:2|lung:11|unk:1</t>
         </is>
@@ -15931,7 +15931,7 @@
         <v>6.55</v>
       </c>
       <c r="F44" s="6" t="n"/>
-      <c r="G44" t="inlineStr">
+      <c r="G44" s="0" t="inlineStr">
         <is>
           <t>lung:9</t>
         </is>
@@ -15956,7 +15956,7 @@
         <v>9.65</v>
       </c>
       <c r="F45" s="6" t="n"/>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="0" t="inlineStr">
         <is>
           <t>bowel:1|head_neck:1|kidney:1|liver:1|lung:8|unk:1|uterus:1</t>
         </is>
@@ -15981,7 +15981,7 @@
         <v>7.9</v>
       </c>
       <c r="F46" s="6" t="n"/>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="0" t="inlineStr">
         <is>
           <t>stomach:1|liver:1|lung:8</t>
         </is>
@@ -16006,7 +16006,7 @@
         <v>9.699999999999999</v>
       </c>
       <c r="F47" s="6" t="n"/>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="0" t="inlineStr">
         <is>
           <t>lung:12|unk:1|uterus:1</t>
         </is>
@@ -16031,7 +16031,7 @@
         <v>13.6</v>
       </c>
       <c r="F48" s="6" t="n"/>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bowel:1|breast:1|stomach:1|head_neck:1|lung:11|unk:2|uterus:2</t>
         </is>
@@ -16056,7 +16056,7 @@
         <v>10.7</v>
       </c>
       <c r="F49" s="6" t="n"/>
-      <c r="G49" t="inlineStr">
+      <c r="G49" s="0" t="inlineStr">
         <is>
           <t>lung:8</t>
         </is>
@@ -16081,7 +16081,7 @@
         <v>12.4</v>
       </c>
       <c r="F50" s="6" t="n"/>
-      <c r="G50" t="inlineStr">
+      <c r="G50" s="0" t="inlineStr">
         <is>
           <t>stomach:1|lung:10|skin:1|unk:2|uterus:2</t>
         </is>
@@ -16110,7 +16110,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G51" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bladder:1|stomach:1|head_neck:2|lung:6|pancreas:1|unk:2|uterus:1</t>
         </is>
@@ -16135,7 +16135,7 @@
         <v>16.2</v>
       </c>
       <c r="F52" s="6" t="n"/>
-      <c r="G52" t="inlineStr">
+      <c r="G52" s="0" t="inlineStr">
         <is>
           <t>lung:8|ovary:1|uterus:1</t>
         </is>
@@ -16160,7 +16160,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="F53" s="6" t="n"/>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="0" t="inlineStr">
         <is>
           <t>lung:9|unk:1|uterus:1</t>
         </is>
@@ -16185,7 +16185,7 @@
         <v>9.699999999999999</v>
       </c>
       <c r="F54" s="6" t="n"/>
-      <c r="G54" t="inlineStr">
+      <c r="G54" s="0" t="inlineStr">
         <is>
           <t>lung:9</t>
         </is>
@@ -16214,7 +16214,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G55" s="0" t="inlineStr">
         <is>
           <t>bowel:7|breast:1|cervix:1|brain:2|stomach:1|lung:1|blood:2|pancreas:1|prostate:1|uterus:1</t>
         </is>
@@ -16243,7 +16243,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G56" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:7|breast:2|stomach:1|prostate:2|uterus:3</t>
         </is>
@@ -16268,7 +16268,7 @@
         <v>6.6</v>
       </c>
       <c r="F57" s="6" t="n"/>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="0" t="inlineStr">
         <is>
           <t>cervix:2|stomach:1|ovary:2|uterus:13</t>
         </is>
@@ -16293,7 +16293,7 @@
         <v>18</v>
       </c>
       <c r="F58" s="6" t="n"/>
-      <c r="G58" t="inlineStr">
+      <c r="G58" s="0" t="inlineStr">
         <is>
           <t>breast:1|lung:1|blood:1|skin:1|unk:1|uterus:8</t>
         </is>
@@ -16322,7 +16322,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G59" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:2|kidney:2|lung:4|uterus:2</t>
         </is>
@@ -16347,7 +16347,7 @@
         <v>4.4</v>
       </c>
       <c r="F60" s="6" t="n"/>
-      <c r="G60" t="inlineStr">
+      <c r="G60" s="0" t="inlineStr">
         <is>
           <t>bowel:5|kidney:1|skin:1</t>
         </is>
@@ -16376,7 +16376,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G61" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:2|breast:1|stomach:1|kidney:1|testis:1</t>
         </is>
@@ -16405,7 +16405,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G62" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:3|breast:1|cervix:1|kidney:1|skin:1|thyroid:1</t>
         </is>
@@ -16430,7 +16430,7 @@
         <v>11.85</v>
       </c>
       <c r="F63" s="6" t="n"/>
-      <c r="G63" t="inlineStr">
+      <c r="G63" s="0" t="inlineStr">
         <is>
           <t>blood:4|ovary:1|uterus:9</t>
         </is>
@@ -16455,7 +16455,7 @@
         <v>7.9</v>
       </c>
       <c r="F64" s="6" t="n"/>
-      <c r="G64" t="inlineStr">
+      <c r="G64" s="0" t="inlineStr">
         <is>
           <t>bowel:1|brain:4|stomach:1|skin:1</t>
         </is>
@@ -16480,7 +16480,7 @@
         <v>12.7</v>
       </c>
       <c r="F65" s="6" t="n"/>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="0" t="inlineStr">
         <is>
           <t>bone:1|bowel:1|brain:6|stomach:4|head_neck:2|lung:1|uterus:1|vulva:1</t>
         </is>
@@ -16509,7 +16509,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G66" s="0" t="inlineStr">
         <is>
           <t>cervix:1|stomach:1|lung:1|blood:1|pleura:1|skin:2</t>
         </is>
@@ -16538,7 +16538,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G67" s="0" t="inlineStr">
         <is>
           <t>breast:1|prostate:1|soft_tissue:1|thyroid:1|uterus:3</t>
         </is>
@@ -16563,7 +16563,7 @@
         <v>14.8</v>
       </c>
       <c r="F68" s="6" t="n"/>
-      <c r="G68" t="inlineStr">
+      <c r="G68" s="0" t="inlineStr">
         <is>
           <t>bladder:2|bowel:5|cervix:1|brain:1|head_neck:1|liver:1|pancreas:1|uterus:1</t>
         </is>
@@ -16588,7 +16588,7 @@
         <v>6.4</v>
       </c>
       <c r="F69" s="6" t="n"/>
-      <c r="G69" t="inlineStr">
+      <c r="G69" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:4|lung:1|uterus:3</t>
         </is>
@@ -16613,7 +16613,7 @@
         <v>5.95</v>
       </c>
       <c r="F70" s="6" t="n"/>
-      <c r="G70" t="inlineStr">
+      <c r="G70" s="0" t="inlineStr">
         <is>
           <t>bladder:3|bowel:2|breast:10|cervix:1|brain:1|head_neck:1|lung:2|soft_tissue:1|uterus:4</t>
         </is>
@@ -16642,7 +16642,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
+      <c r="G71" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:1|brain:1|ovary:1|uterus:5</t>
         </is>
@@ -16667,7 +16667,7 @@
         <v>6.9</v>
       </c>
       <c r="F72" s="6" t="n"/>
-      <c r="G72" t="inlineStr">
+      <c r="G72" s="0" t="inlineStr">
         <is>
           <t>bowel:3|breast:3|skin:1|uterus:5</t>
         </is>
@@ -16696,7 +16696,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G73" s="0" t="inlineStr">
         <is>
           <t>bowel:1|brain:2|lung:1|soft_tissue:2|uterus:3</t>
         </is>
@@ -16725,7 +16725,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
+      <c r="G74" s="0" t="inlineStr">
         <is>
           <t>bladder:1|breast:2|brain:1|lung:1|uterus:1</t>
         </is>
@@ -16754,7 +16754,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G75" s="0" t="inlineStr">
         <is>
           <t>bowel:3|brain:3|stomach:2|prostate:2|uterus:4</t>
         </is>
@@ -16783,7 +16783,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G76" s="0" t="inlineStr">
         <is>
           <t>lung:3|prostate:3|uterus:1</t>
         </is>
@@ -16808,7 +16808,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="F77" s="6" t="n"/>
-      <c r="G77" t="inlineStr">
+      <c r="G77" s="0" t="inlineStr">
         <is>
           <t>stomach:1|ovary:2|skin:1|uterus:9</t>
         </is>
@@ -16837,7 +16837,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr">
+      <c r="G78" s="0" t="inlineStr">
         <is>
           <t>bowel:1|cervix:1|liver:1|ovary:2|uterus:17</t>
         </is>
@@ -16862,7 +16862,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="F79" s="6" t="n"/>
-      <c r="G79" t="inlineStr">
+      <c r="G79" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:2|cervix:1|brain:3|head_neck:1|liver:1|blood:1|soft_tissue:1|thyroid:1|uterus:5</t>
         </is>
@@ -16891,7 +16891,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr">
+      <c r="G80" s="0" t="inlineStr">
         <is>
           <t>breast:1|brain:1|soft_tissue:1|prostate:1|unk:2|uterus:1</t>
         </is>
@@ -16920,7 +16920,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
+      <c r="G81" s="0" t="inlineStr">
         <is>
           <t>bladder:1|breast:1|brain:7|stomach:2|head_neck:1|lung:1|blood:1|prostate:2|soft_tissue:1|uterus:6</t>
         </is>
@@ -16949,7 +16949,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
+      <c r="G82" s="0" t="inlineStr">
         <is>
           <t>breast:1|cervix:1|brain:1|lung:2|prostate:1|soft_tissue:1|unk:1|uterus:3</t>
         </is>
@@ -16978,7 +16978,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="G83" s="0" t="inlineStr">
         <is>
           <t>bowel:1|brain:4|skin:2|testis:1|uterus:3</t>
         </is>
@@ -17007,7 +17007,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G84" s="0" t="inlineStr">
         <is>
           <t>bowel:2|brain:1|stomach:1|kidney:1|lung:1|uterus:4</t>
         </is>
@@ -17036,7 +17036,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
+      <c r="G85" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:2|cervix:1|brain:6|lung:3|uterus:2</t>
         </is>
@@ -17065,7 +17065,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G86" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:2|brain:1|pancreas:1|skin:2|uterus:1</t>
         </is>
@@ -17090,7 +17090,7 @@
         <v>14.6</v>
       </c>
       <c r="F87" s="6" t="n"/>
-      <c r="G87" t="inlineStr">
+      <c r="G87" s="0" t="inlineStr">
         <is>
           <t>brain:2|prostate:2|skin:1|unk:1|uterus:1</t>
         </is>
@@ -17119,7 +17119,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr">
+      <c r="G88" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:3|brain:2|lung:2|ovary:1|penis:1|prostate:1|uterus:4</t>
         </is>
@@ -17148,7 +17148,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
+      <c r="G89" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:1|lung:1|skin:1|uterus:6</t>
         </is>
@@ -17177,7 +17177,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr">
+      <c r="G90" s="0" t="inlineStr">
         <is>
           <t>bladder:1|breast:2|head_neck:1|lung:3|prostate:2|skin:1|uterus:4</t>
         </is>
@@ -17202,7 +17202,7 @@
         <v>13.2</v>
       </c>
       <c r="F91" s="6" t="n"/>
-      <c r="G91" t="inlineStr">
+      <c r="G91" s="0" t="inlineStr">
         <is>
           <t>bowel:1|breast:2|head_neck:1|uterus:7</t>
         </is>
@@ -17227,7 +17227,7 @@
         <v>10.15</v>
       </c>
       <c r="F92" s="6" t="n"/>
-      <c r="G92" t="inlineStr">
+      <c r="G92" s="0" t="inlineStr">
         <is>
           <t>kidney:1|ovary:1|pancreas:1|uterus:4</t>
         </is>
@@ -17256,7 +17256,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr">
+      <c r="G93" s="0" t="inlineStr">
         <is>
           <t>bone:1|brain:3|stomach:1|head_neck:1|blood:1|thyroid:1|uterus:2</t>
         </is>
@@ -17281,7 +17281,7 @@
         <v>9.25</v>
       </c>
       <c r="F94" s="6" t="n"/>
-      <c r="G94" t="inlineStr">
+      <c r="G94" s="0" t="inlineStr">
         <is>
           <t>bowel:2|brain:3|skin:1|uterus:4</t>
         </is>
@@ -17310,7 +17310,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr">
+      <c r="G95" s="0" t="inlineStr">
         <is>
           <t>breast:1|cervix:1|brain:3|head_neck:1|thyroid:1|uterus:3</t>
         </is>
@@ -17335,7 +17335,7 @@
         <v>5.25</v>
       </c>
       <c r="F96" s="6" t="n"/>
-      <c r="G96" t="inlineStr">
+      <c r="G96" s="0" t="inlineStr">
         <is>
           <t>bowel:1|brain:2|kidney:1|lung:1|blood:1|prostate:1|uterus:4</t>
         </is>
@@ -17364,7 +17364,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr">
+      <c r="G97" s="0" t="inlineStr">
         <is>
           <t>brain:4|kidney:1|lung:2|ovary:1|prostate:1|uterus:3</t>
         </is>
@@ -17393,7 +17393,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr">
+      <c r="G98" s="0" t="inlineStr">
         <is>
           <t>bowel:1|brain:4|stomach:1|head_neck:1|lung:1|blood:6|testis:1</t>
         </is>
@@ -17418,7 +17418,7 @@
         <v>13.6</v>
       </c>
       <c r="F99" s="6" t="n"/>
-      <c r="G99" t="inlineStr">
+      <c r="G99" s="0" t="inlineStr">
         <is>
           <t>bowel:2|cervix:1|brain:2|stomach:3|lung:1|ovary:1|prostate:1|skin:3|soft_tissue:1|uterus:2</t>
         </is>
@@ -17443,7 +17443,7 @@
         <v>10.5</v>
       </c>
       <c r="F100" s="6" t="n"/>
-      <c r="G100" t="inlineStr">
+      <c r="G100" s="0" t="inlineStr">
         <is>
           <t>bowel:6|head_neck:1|lung:3|blood:1|skin:1|uterus:2</t>
         </is>
@@ -17472,9 +17472,9 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>ampullaofvater:1|biliary_tract:1|bladder:1|bowel:1|liver:1|lung:2|skin:1|unk:1|uterus:1</t>
+      <c r="G101" s="0" t="inlineStr">
+        <is>
+          <t>ampulla_of_vater:1|biliary_tract:1|bladder:1|bowel:1|liver:1|lung:2|skin:1|unk:1|uterus:1</t>
         </is>
       </c>
     </row>
@@ -17497,7 +17497,7 @@
         <v>7.9</v>
       </c>
       <c r="F102" s="6" t="n"/>
-      <c r="G102" t="inlineStr">
+      <c r="G102" s="0" t="inlineStr">
         <is>
           <t>bladder:1|stomach:1|lung:3|pancreas:1|prostate:1|soft_tissue:1|uterus:1</t>
         </is>
@@ -17526,7 +17526,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
+      <c r="G103" s="0" t="inlineStr">
         <is>
           <t>adrenal_gland:2|bladder:2|bowel:1|brain:1|stomach:1|eye:1|kidney:1|lung:1|blood:1|pancreas:1|prostate:1|soft_tissue:1|unk:2</t>
         </is>
@@ -17555,7 +17555,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr">
+      <c r="G104" s="0" t="inlineStr">
         <is>
           <t>thyroid:3</t>
         </is>
@@ -17584,7 +17584,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr">
+      <c r="G105" s="0" t="inlineStr">
         <is>
           <t>breast:4|cervix:1|brain:2|stomach:1|kidney:1|ovary:1|prostate:2|testis:9|uterus:13|vulva:1</t>
         </is>
@@ -17609,7 +17609,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="F106" s="6" t="n"/>
-      <c r="G106" t="inlineStr">
+      <c r="G106" s="0" t="inlineStr">
         <is>
           <t>bowel:2|brain:1|head_neck:1|lung:1|ovary:2|uterus:12</t>
         </is>
@@ -17638,7 +17638,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr">
+      <c r="G107" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:3|blood:2|ovary:1|pancreas:1|prostate:1|uterus:8</t>
         </is>
@@ -17663,7 +17663,7 @@
         <v>19</v>
       </c>
       <c r="F108" s="6" t="n"/>
-      <c r="G108" t="inlineStr">
+      <c r="G108" s="0" t="inlineStr">
         <is>
           <t>bladder:1|brain:1|stomach:1|kidney:2|liver:1|lung:3</t>
         </is>
@@ -17688,7 +17688,7 @@
         <v>7.5</v>
       </c>
       <c r="F109" s="6" t="n"/>
-      <c r="G109" t="inlineStr">
+      <c r="G109" s="0" t="inlineStr">
         <is>
           <t>bowel:5|skin:1</t>
         </is>
@@ -17717,7 +17717,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr">
+      <c r="G110" s="0" t="inlineStr">
         <is>
           <t>bowel:6|lung:1|prostate:1</t>
         </is>
@@ -17742,7 +17742,7 @@
         <v>11.4</v>
       </c>
       <c r="F111" s="6" t="n"/>
-      <c r="G111" t="inlineStr">
+      <c r="G111" s="0" t="inlineStr">
         <is>
           <t>bowel:7</t>
         </is>
@@ -17767,7 +17767,7 @@
         <v>9.699999999999999</v>
       </c>
       <c r="F112" s="6" t="n"/>
-      <c r="G112" t="inlineStr">
+      <c r="G112" s="0" t="inlineStr">
         <is>
           <t>bowel:4|lung:1|ovary:1|pancreas:2|uterus:1</t>
         </is>
@@ -17792,7 +17792,7 @@
         <v>6.1</v>
       </c>
       <c r="F113" s="6" t="n"/>
-      <c r="G113" t="inlineStr">
+      <c r="G113" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:2|bowel:4</t>
         </is>
@@ -17817,7 +17817,7 @@
         <v>5.3</v>
       </c>
       <c r="F114" s="6" t="n"/>
-      <c r="G114" t="inlineStr">
+      <c r="G114" s="0" t="inlineStr">
         <is>
           <t>bowel:6|breast:1|lung:1|blood:1|pancreas:1|unk:1</t>
         </is>
@@ -17842,9 +17842,9 @@
         <v>5.3</v>
       </c>
       <c r="F115" s="6" t="n"/>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>ampullaofvater:1|biliary_tract:1|bowel:1|stomach:2|lung:1|pancreas:4|uterus:1</t>
+      <c r="G115" s="0" t="inlineStr">
+        <is>
+          <t>ampulla_of_vater:1|biliary_tract:1|bowel:1|stomach:2|lung:1|pancreas:4|uterus:1</t>
         </is>
       </c>
     </row>
@@ -17867,7 +17867,7 @@
         <v>7</v>
       </c>
       <c r="F116" s="6" t="n"/>
-      <c r="G116" t="inlineStr">
+      <c r="G116" s="0" t="inlineStr">
         <is>
           <t>bowel:11|stomach:2|kidney:1|lung:1|blood:1|pancreas:1|uterus:1</t>
         </is>
@@ -17896,7 +17896,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
+      <c r="G117" s="0" t="inlineStr">
         <is>
           <t>bowel:4|breast:1|lung:3|uterus:1</t>
         </is>
@@ -17925,7 +17925,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr">
+      <c r="G118" s="0" t="inlineStr">
         <is>
           <t>bowel:10|cervix:1|pancreas:4|uterus:2</t>
         </is>
@@ -17954,7 +17954,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr">
+      <c r="G119" s="0" t="inlineStr">
         <is>
           <t>bowel:4|breast:2|lung:1|pancreas:2</t>
         </is>
@@ -17979,9 +17979,9 @@
         <v>6.1</v>
       </c>
       <c r="F120" s="6" t="n"/>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>ampullaofvater:1|bowel:4|lung:1|pancreas:2|unk:1</t>
+      <c r="G120" s="0" t="inlineStr">
+        <is>
+          <t>ampulla_of_vater:1|bowel:4|lung:1|pancreas:2|unk:1</t>
         </is>
       </c>
     </row>
@@ -18004,7 +18004,7 @@
         <v>13.9</v>
       </c>
       <c r="F121" s="6" t="n"/>
-      <c r="G121" t="inlineStr">
+      <c r="G121" s="0" t="inlineStr">
         <is>
           <t>bowel:1|stomach:2|lung:5|skin:1|uterus:1</t>
         </is>
@@ -18029,7 +18029,7 @@
         <v>7.9</v>
       </c>
       <c r="F122" s="6" t="n"/>
-      <c r="G122" t="inlineStr">
+      <c r="G122" s="0" t="inlineStr">
         <is>
           <t>brain:2|stomach:2|lung:3|pancreas:1|skin:1|uterus:5</t>
         </is>
@@ -18054,7 +18054,7 @@
         <v>7.9</v>
       </c>
       <c r="F123" s="6" t="n"/>
-      <c r="G123" t="inlineStr">
+      <c r="G123" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|stomach:1|lung:5|ovary:1|pancreas:1</t>
         </is>
@@ -18083,7 +18083,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr">
+      <c r="G124" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:1|brain:1|stomach:1|lung:2|pancreas:1|skin:1|uterus:4</t>
         </is>
@@ -18112,7 +18112,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr">
+      <c r="G125" s="0" t="inlineStr">
         <is>
           <t>adrenal_gland:1|bladder:1|breast:1|cervix:1|blood:1|ovary:6|uterus:4</t>
         </is>
@@ -18141,7 +18141,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr">
+      <c r="G126" s="0" t="inlineStr">
         <is>
           <t>breast:2|stomach:1|head_neck:1|ovary:2|thyroid:1|unk:1|uterus:9</t>
         </is>
@@ -18170,7 +18170,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr">
+      <c r="G127" s="0" t="inlineStr">
         <is>
           <t>ovary:1|unk:1|uterus:5</t>
         </is>
@@ -18195,7 +18195,7 @@
         <v>2.2</v>
       </c>
       <c r="F128" s="6" t="n"/>
-      <c r="G128" t="inlineStr">
+      <c r="G128" s="0" t="inlineStr">
         <is>
           <t>blood:1|prostate:4|unk:1|uterus:2</t>
         </is>
@@ -18224,7 +18224,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr">
+      <c r="G129" s="0" t="inlineStr">
         <is>
           <t>bladder:4|breast:1|blood:2|pancreas:1|prostate:6|skin:1|soft_tissue:1</t>
         </is>
@@ -18249,7 +18249,7 @@
         <v>6.1</v>
       </c>
       <c r="F130" s="6" t="n"/>
-      <c r="G130" t="inlineStr">
+      <c r="G130" s="0" t="inlineStr">
         <is>
           <t>cervix:1|lung:12|pancreas:1|unk:1</t>
         </is>
@@ -18274,7 +18274,7 @@
         <v>7</v>
       </c>
       <c r="F131" s="6" t="n"/>
-      <c r="G131" t="inlineStr">
+      <c r="G131" s="0" t="inlineStr">
         <is>
           <t>cervix:1|lung:7|unk:1</t>
         </is>
@@ -18303,7 +18303,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr">
+      <c r="G132" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|breast:1|cervix:2|lung:7|unk:1</t>
         </is>
@@ -18328,7 +18328,7 @@
         <v>7.45</v>
       </c>
       <c r="F133" s="6" t="n"/>
-      <c r="G133" t="inlineStr">
+      <c r="G133" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bowel:12|stomach:1</t>
         </is>
@@ -18353,7 +18353,7 @@
         <v>7</v>
       </c>
       <c r="F134" s="6" t="n"/>
-      <c r="G134" t="inlineStr">
+      <c r="G134" s="0" t="inlineStr">
         <is>
           <t>bowel:21|lung:1</t>
         </is>
@@ -18378,7 +18378,7 @@
         <v>6.9</v>
       </c>
       <c r="F135" s="6" t="n"/>
-      <c r="G135" t="inlineStr">
+      <c r="G135" s="0" t="inlineStr">
         <is>
           <t>bowel:11|blood:2</t>
         </is>
@@ -18403,7 +18403,7 @@
         <v>6.1</v>
       </c>
       <c r="F136" s="6" t="n"/>
-      <c r="G136" t="inlineStr">
+      <c r="G136" s="0" t="inlineStr">
         <is>
           <t>bowel:6</t>
         </is>
@@ -18428,7 +18428,7 @@
         <v>4.9</v>
       </c>
       <c r="F137" s="6" t="n"/>
-      <c r="G137" t="inlineStr">
+      <c r="G137" s="0" t="inlineStr">
         <is>
           <t>bowel:6|uterus:1</t>
         </is>
@@ -18453,7 +18453,7 @@
         <v>7.9</v>
       </c>
       <c r="F138" s="6" t="n"/>
-      <c r="G138" t="inlineStr">
+      <c r="G138" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bowel:6|stomach:3|lung:1|pancreas:1|unk:1</t>
         </is>
@@ -18478,7 +18478,7 @@
         <v>4.25</v>
       </c>
       <c r="F139" s="6" t="n"/>
-      <c r="G139" t="inlineStr">
+      <c r="G139" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bladder:1|bowel:1|breast:1|stomach:1|head_neck:2|liver:1|lung:5|ovary:1|pancreas:1|skin:1</t>
         </is>
@@ -18503,7 +18503,7 @@
         <v>4.4</v>
       </c>
       <c r="F140" s="6" t="n"/>
-      <c r="G140" t="inlineStr">
+      <c r="G140" s="0" t="inlineStr">
         <is>
           <t>bowel:5|breast:4|brain:4|stomach:2|head_neck:1|kidney:1|liver:1|lung:7|ovary:2|pancreas:2|prostate:1|skin:2|soft_tissue:2|unk:1|uterus:1|vulva:1</t>
         </is>
@@ -18528,7 +18528,7 @@
         <v>7</v>
       </c>
       <c r="F141" s="6" t="n"/>
-      <c r="G141" t="inlineStr">
+      <c r="G141" s="0" t="inlineStr">
         <is>
           <t>bladder:2|bone:1|breast:2|stomach:2|head_neck:1|liver:3|lung:5|blood:3|prostate:1|uterus:1</t>
         </is>
@@ -18557,7 +18557,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr">
+      <c r="G142" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bone:1|bowel:6|breast:3|cervix:1|brain:1|stomach:2|liver:2|lung:4|blood:1|ovary:2|pancreas:2|prostate:2|unk:1|uterus:1</t>
         </is>
@@ -18582,7 +18582,7 @@
         <v>5.1</v>
       </c>
       <c r="F143" s="6" t="n"/>
-      <c r="G143" t="inlineStr">
+      <c r="G143" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bladder:1|bowel:1|brain:2|stomach:1|lung:2|ovary:1|pancreas:1|uterus:2</t>
         </is>
@@ -18611,7 +18611,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr">
+      <c r="G144" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bladder:3|bowel:2|breast:4|brain:4|head_neck:1|liver:2|lung:14|ovary:2|pancreas:1|soft_tissue:2|uterus:1</t>
         </is>
@@ -18640,7 +18640,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr">
+      <c r="G145" s="0" t="inlineStr">
         <is>
           <t>bowel:2|stomach:3|liver:1|lung:5|blood:3|pancreas:2|prostate:1|skin:1|thyroid:1|unk:1|uterus:1</t>
         </is>
@@ -18665,7 +18665,7 @@
         <v>6.75</v>
       </c>
       <c r="F146" s="6" t="n"/>
-      <c r="G146" t="inlineStr">
+      <c r="G146" s="0" t="inlineStr">
         <is>
           <t>biliary_tract:1|bowel:1|breast:2|stomach:2|liver:4|lung:2|blood:1|soft_tissue:1|unk:1|uterus:1</t>
         </is>
@@ -18690,7 +18690,7 @@
         <v>5.3</v>
       </c>
       <c r="F147" s="6" t="n"/>
-      <c r="G147" t="inlineStr">
+      <c r="G147" s="0" t="inlineStr">
         <is>
           <t>breast:2|brain:3|stomach:1|lung:4|blood:1|ovary:2|pancreas:1|prostate:2|skin:6|unk:3</t>
         </is>
@@ -18719,7 +18719,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr">
+      <c r="G148" s="0" t="inlineStr">
         <is>
           <t>bladder:7|bowel:1|breast:9|stomach:1|head_neck:1|lung:13|ovary:2|pancreas:1|prostate:2|testis:1</t>
         </is>
@@ -18748,7 +18748,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr">
+      <c r="G149" s="0" t="inlineStr">
         <is>
           <t>bladder:2|bowel:7|breast:8|brain:4|head_neck:1|liver:1|lung:13|blood:2|ovary:2|pancreas:2|prostate:4|skin:2|soft_tissue:2|testis:1|unk:1|uterus:1</t>
         </is>
@@ -18773,7 +18773,7 @@
         <v>5.6</v>
       </c>
       <c r="F150" s="6" t="n"/>
-      <c r="G150" t="inlineStr">
+      <c r="G150" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:6|brain:1|head_neck:1|liver:1|lung:4|pancreas:1|skin:1|soft_tissue:1|uterus:2</t>
         </is>
@@ -18798,7 +18798,7 @@
         <v>5.8</v>
       </c>
       <c r="F151" s="6" t="n"/>
-      <c r="G151" t="inlineStr">
+      <c r="G151" s="0" t="inlineStr">
         <is>
           <t>bladder:2|bowel:5|breast:4|brain:3|stomach:2|head_neck:2|kidney:1|liver:1|lung:12|blood:1|ovary:1|pancreas:2|skin:1|soft_tissue:3|unk:1|uterus:1</t>
         </is>
@@ -18827,7 +18827,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr">
+      <c r="G152" s="0" t="inlineStr">
         <is>
           <t>bowel:2|brain:3|lung:5|blood:2|pancreas:2|prostate:5|unk:1|uterus:3</t>
         </is>
@@ -18852,7 +18852,7 @@
         <v>5.3</v>
       </c>
       <c r="F153" s="6" t="n"/>
-      <c r="G153" t="inlineStr">
+      <c r="G153" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:2|breast:1|stomach:3|head_neck:1|liver:3|lung:3|blood:1|ovary:2|prostate:3|skin:1|uterus:4</t>
         </is>
@@ -18877,9 +18877,9 @@
         <v>6.1</v>
       </c>
       <c r="F154" s="6" t="n"/>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>ampullaofvater:1|bowel:1|breast:2|brain:2|stomach:1|head_neck:2|liver:2|lung:12|blood:1|ovary:2|pleura:1|thyroid:1|unk:1|uterus:3|vulva:1</t>
+      <c r="G154" s="0" t="inlineStr">
+        <is>
+          <t>ampulla_of_vater:1|bowel:1|breast:2|brain:2|stomach:1|head_neck:2|liver:2|lung:12|blood:1|ovary:2|pleura:1|thyroid:1|unk:1|uterus:3|vulva:1</t>
         </is>
       </c>
     </row>
@@ -18902,7 +18902,7 @@
         <v>7</v>
       </c>
       <c r="F155" s="6" t="n"/>
-      <c r="G155" t="inlineStr">
+      <c r="G155" s="0" t="inlineStr">
         <is>
           <t>bladder:3|breast:2|brain:4|stomach:1|lung:4|ovary:5|prostate:2|skin:3|uterus:3|vulva:1</t>
         </is>
@@ -18931,9 +18931,9 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>ampullaofvater:1|bladder:3|bowel:3|breast:2|brain:1|stomach:1|head_neck:5|lung:11|ovary:1|pancreas:2|unk:4|uterus:3|vulva:1</t>
+      <c r="G156" s="0" t="inlineStr">
+        <is>
+          <t>ampulla_of_vater:1|bladder:3|bowel:3|breast:2|brain:1|stomach:1|head_neck:5|lung:11|ovary:1|pancreas:2|unk:4|uterus:3|vulva:1</t>
         </is>
       </c>
     </row>
@@ -18960,7 +18960,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr">
+      <c r="G157" s="0" t="inlineStr">
         <is>
           <t>bladder:2|bowel:1|breast:3|lung:1|blood:3|skin:3|thyroid:2|unk:1</t>
         </is>
@@ -18989,7 +18989,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G158" t="inlineStr">
+      <c r="G158" s="0" t="inlineStr">
         <is>
           <t>breast:1|liver:1|lung:5|skin:4</t>
         </is>
@@ -19014,7 +19014,7 @@
         <v>9.9</v>
       </c>
       <c r="F159" s="6" t="n"/>
-      <c r="G159" t="inlineStr">
+      <c r="G159" s="0" t="inlineStr">
         <is>
           <t>breast:2|stomach:2|kidney:1|lung:12|testis:1|unk:1|uterus:1</t>
         </is>
@@ -19043,7 +19043,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr">
+      <c r="G160" s="0" t="inlineStr">
         <is>
           <t>brain:1|head_neck:1|liver:1|lung:1|pleura:1|testis:1|unk:1|uterus:1</t>
         </is>
@@ -19072,7 +19072,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr">
+      <c r="G161" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:1|lung:2|pancreas:1|prostate:1</t>
         </is>
@@ -19101,7 +19101,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G162" t="inlineStr">
+      <c r="G162" s="0" t="inlineStr">
         <is>
           <t>bowel:2|breast:2|brain:1|lung:1|unk:1|uterus:1</t>
         </is>
@@ -19130,7 +19130,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G163" t="inlineStr">
+      <c r="G163" s="0" t="inlineStr">
         <is>
           <t>bladder:1|bowel:1|breast:1|cervix:1|lung:1|blood:3|ovary:2|pancreas:1|skin:1|uterus:1</t>
         </is>
@@ -19159,7 +19159,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G164" t="inlineStr">
+      <c r="G164" s="0" t="inlineStr">
         <is>
           <t>adrenal_gland:1|kidney:4|pancreas:2|prostate:1|soft_tissue:1|thyroid:1|uterus:1</t>
         </is>
@@ -19188,7 +19188,7 @@
           <t>OncoKB</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr">
+      <c r="G165" s="0" t="inlineStr">
         <is>
           <t>kidney:8</t>
         </is>

</xml_diff>